<commit_message>
Add media key controls
</commit_message>
<xml_diff>
--- a/Key layout.xlsx
+++ b/Key layout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Github\Keyboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077B3B91-EF39-41C5-8747-4842B3905FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0F2640-C959-4208-A4FF-354C488EB51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5980" yWindow="1720" windowWidth="30890" windowHeight="18330" xr2:uid="{8FB76BC3-2A3C-4BB8-828D-89A98B45AE68}"/>
+    <workbookView xWindow="7510" yWindow="290" windowWidth="30890" windowHeight="18330" xr2:uid="{8FB76BC3-2A3C-4BB8-828D-89A98B45AE68}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="101">
   <si>
     <t>A</t>
   </si>
@@ -329,6 +329,15 @@
   </si>
   <si>
     <t>Space</t>
+  </si>
+  <si>
+    <t>⏯</t>
+  </si>
+  <si>
+    <t>⏮</t>
+  </si>
+  <si>
+    <t>⏭</t>
   </si>
 </sst>
 </file>
@@ -912,7 +921,9 @@
     </row>
     <row r="5" spans="2:35" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C5" s="6"/>
-      <c r="D5" s="19"/>
+      <c r="D5" s="19" t="s">
+        <v>100</v>
+      </c>
       <c r="E5" s="9" t="s">
         <v>54</v>
       </c>
@@ -1033,7 +1044,9 @@
     </row>
     <row r="7" spans="2:35" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C7" s="6"/>
-      <c r="D7" s="19"/>
+      <c r="D7" s="19" t="s">
+        <v>98</v>
+      </c>
       <c r="E7" s="9" t="s">
         <v>66</v>
       </c>
@@ -1142,7 +1155,9 @@
       </c>
     </row>
     <row r="9" spans="2:35" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D9" s="19"/>
+      <c r="D9" s="19" t="s">
+        <v>99</v>
+      </c>
       <c r="E9" s="9"/>
       <c r="F9" s="4" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Add the ² key (POW_2) to accentLayer2 on Z
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: 490315b3-83c0-4fe2-83a8-3d9bd83c6f8c
</commit_message>
<xml_diff>
--- a/Key layout.xlsx
+++ b/Key layout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Github\Keyboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\copilot-workspace\sessions\add-power-2\worktree\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0F2640-C959-4208-A4FF-354C488EB51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49AC69BE-C321-4BC1-BB99-C7861C0A9A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7510" yWindow="290" windowWidth="30890" windowHeight="18330" xr2:uid="{8FB76BC3-2A3C-4BB8-828D-89A98B45AE68}"/>
+    <workbookView xWindow="8500" yWindow="1880" windowWidth="26710" windowHeight="17190" xr2:uid="{8FB76BC3-2A3C-4BB8-828D-89A98B45AE68}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="102">
   <si>
     <t>A</t>
   </si>
@@ -338,6 +338,9 @@
   </si>
   <si>
     <t>⏭</t>
+  </si>
+  <si>
+    <t>²</t>
   </si>
 </sst>
 </file>
@@ -874,7 +877,9 @@
       <c r="AC3" s="6"/>
     </row>
     <row r="4" spans="2:35" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="F4" s="19"/>
+      <c r="F4" s="19" t="s">
+        <v>101</v>
+      </c>
       <c r="G4" s="9" t="s">
         <v>55</v>
       </c>

</xml_diff>